<commit_message>
new econ moniotoring program
</commit_message>
<xml_diff>
--- a/99_economic/Z.economic_pulse_monthly/pce_detail.xlsx
+++ b/99_economic/Z.economic_pulse_monthly/pce_detail.xlsx
@@ -1456,7 +1456,7 @@
         <v>6</v>
       </c>
       <c r="I20" t="n">
-        <v>201495</v>
+        <v>199022</v>
       </c>
       <c r="J20" t="inlineStr">
         <is>
@@ -1464,10 +1464,10 @@
         </is>
       </c>
       <c r="K20" t="n">
-        <v>0.03949669571138936</v>
+        <v>0.02673868519750933</v>
       </c>
       <c r="L20" t="n">
-        <v>43</v>
+        <v>35</v>
       </c>
     </row>
     <row r="21">
@@ -2436,7 +2436,7 @@
         <v>6</v>
       </c>
       <c r="I39" t="n">
-        <v>187528</v>
+        <v>187440</v>
       </c>
       <c r="J39" t="inlineStr">
         <is>
@@ -2444,7 +2444,7 @@
         </is>
       </c>
       <c r="K39" t="n">
-        <v>0.1147716396882672</v>
+        <v>0.1142485183181647</v>
       </c>
       <c r="L39" t="n">
         <v>87</v>
@@ -3416,7 +3416,7 @@
         <v>6</v>
       </c>
       <c r="I58" t="n">
-        <v>228784</v>
+        <v>228872</v>
       </c>
       <c r="J58" t="inlineStr">
         <is>
@@ -3424,10 +3424,10 @@
         </is>
       </c>
       <c r="K58" t="n">
-        <v>0.03034970388885139</v>
+        <v>0.03074601995091086</v>
       </c>
       <c r="L58" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="59">
@@ -4396,7 +4396,7 @@
         <v>6</v>
       </c>
       <c r="I77" t="n">
-        <v>88121</v>
+        <v>88109</v>
       </c>
       <c r="J77" t="inlineStr">
         <is>
@@ -4404,10 +4404,10 @@
         </is>
       </c>
       <c r="K77" t="n">
-        <v>0.02324690254183159</v>
+        <v>0.02310756046865392</v>
       </c>
       <c r="L77" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="78">
@@ -5376,7 +5376,7 @@
         <v>6</v>
       </c>
       <c r="I96" t="n">
-        <v>168824</v>
+        <v>168643</v>
       </c>
       <c r="J96" t="inlineStr">
         <is>
@@ -5384,7 +5384,7 @@
         </is>
       </c>
       <c r="K96" t="n">
-        <v>-0.003800127457691094</v>
+        <v>-0.004868175702787525</v>
       </c>
       <c r="L96" t="n">
         <v>11</v>
@@ -6356,7 +6356,7 @@
         <v>6</v>
       </c>
       <c r="I115" t="n">
-        <v>26090</v>
+        <v>26103</v>
       </c>
       <c r="J115" t="inlineStr">
         <is>
@@ -6364,10 +6364,10 @@
         </is>
       </c>
       <c r="K115" t="n">
-        <v>0.04289083423272166</v>
+        <v>0.04341048087300625</v>
       </c>
       <c r="L115" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="116">
@@ -7336,7 +7336,7 @@
         <v>6</v>
       </c>
       <c r="I134" t="n">
-        <v>308087</v>
+        <v>309216</v>
       </c>
       <c r="J134" t="inlineStr">
         <is>
@@ -7344,10 +7344,10 @@
         </is>
       </c>
       <c r="K134" t="n">
-        <v>0.01412460993561471</v>
+        <v>0.01784091956444467</v>
       </c>
       <c r="L134" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
     </row>
     <row r="135">
@@ -8316,7 +8316,7 @@
         <v>6</v>
       </c>
       <c r="I153" t="n">
-        <v>187436</v>
+        <v>186442</v>
       </c>
       <c r="J153" t="inlineStr">
         <is>
@@ -8324,10 +8324,10 @@
         </is>
       </c>
       <c r="K153" t="n">
-        <v>0.0813885731758679</v>
+        <v>0.07565381442228358</v>
       </c>
       <c r="L153" t="n">
-        <v>78</v>
+        <v>74</v>
       </c>
     </row>
     <row r="154">
@@ -9296,7 +9296,7 @@
         <v>6</v>
       </c>
       <c r="I172" t="n">
-        <v>2168185</v>
+        <v>2168449</v>
       </c>
       <c r="J172" t="inlineStr">
         <is>
@@ -9304,10 +9304,10 @@
         </is>
       </c>
       <c r="K172" t="n">
-        <v>0.01235736340761795</v>
+        <v>0.01248062887801815</v>
       </c>
       <c r="L172" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
     </row>
     <row r="173">
@@ -10276,7 +10276,7 @@
         <v>6</v>
       </c>
       <c r="I191" t="n">
-        <v>8433</v>
+        <v>8446</v>
       </c>
       <c r="J191" t="inlineStr">
         <is>
@@ -10284,10 +10284,10 @@
         </is>
       </c>
       <c r="K191" t="n">
-        <v>0.0375246062992125</v>
+        <v>0.03912401574803148</v>
       </c>
       <c r="L191" t="n">
-        <v>39</v>
+        <v>43</v>
       </c>
     </row>
     <row r="192">
@@ -11256,7 +11256,7 @@
         <v>6</v>
       </c>
       <c r="I210" t="n">
-        <v>249961</v>
+        <v>248331</v>
       </c>
       <c r="J210" t="inlineStr">
         <is>
@@ -11264,10 +11264,10 @@
         </is>
       </c>
       <c r="K210" t="n">
-        <v>0.01552781152113236</v>
+        <v>0.008905537115207363</v>
       </c>
       <c r="L210" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
     </row>
     <row r="211">
@@ -12236,7 +12236,7 @@
         <v>6</v>
       </c>
       <c r="I229" t="n">
-        <v>314555</v>
+        <v>313038</v>
       </c>
       <c r="J229" t="inlineStr">
         <is>
@@ -12244,10 +12244,10 @@
         </is>
       </c>
       <c r="K229" t="n">
-        <v>0.006740300016962797</v>
+        <v>0.001885107649568507</v>
       </c>
       <c r="L229" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="230">
@@ -13227,7 +13227,7 @@
         <v>0.04966714039943154</v>
       </c>
       <c r="L248" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="249">
@@ -14207,7 +14207,7 @@
         <v>-0.02573099415204683</v>
       </c>
       <c r="L267" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="268">
@@ -15176,7 +15176,7 @@
         <v>6</v>
       </c>
       <c r="I286" t="n">
-        <v>280289</v>
+        <v>280591</v>
       </c>
       <c r="J286" t="inlineStr">
         <is>
@@ -15184,10 +15184,10 @@
         </is>
       </c>
       <c r="K286" t="n">
-        <v>0.01261208534743741</v>
+        <v>0.01370313369316256</v>
       </c>
       <c r="L286" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
     </row>
     <row r="287">
@@ -16156,7 +16156,7 @@
         <v>6</v>
       </c>
       <c r="I305" t="n">
-        <v>18941</v>
+        <v>18947</v>
       </c>
       <c r="J305" t="inlineStr">
         <is>
@@ -16164,10 +16164,10 @@
         </is>
       </c>
       <c r="K305" t="n">
-        <v>0.1188493118317679</v>
+        <v>0.1192037332388209</v>
       </c>
       <c r="L305" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="306">
@@ -17136,7 +17136,7 @@
         <v>6</v>
       </c>
       <c r="I324" t="n">
-        <v>1039679</v>
+        <v>1043718</v>
       </c>
       <c r="J324" t="inlineStr">
         <is>
@@ -17144,7 +17144,7 @@
         </is>
       </c>
       <c r="K324" t="n">
-        <v>0.08445958984340374</v>
+        <v>0.08867255584865874</v>
       </c>
       <c r="L324" t="n">
         <v>80</v>
@@ -18116,7 +18116,7 @@
         <v>6</v>
       </c>
       <c r="I343" t="n">
-        <v>35149</v>
+        <v>35153</v>
       </c>
       <c r="J343" t="inlineStr">
         <is>
@@ -18124,7 +18124,7 @@
         </is>
       </c>
       <c r="K343" t="n">
-        <v>0.07276056767892558</v>
+        <v>0.07288264916831988</v>
       </c>
       <c r="L343" t="n">
         <v>72</v>
@@ -19096,7 +19096,7 @@
         <v>6</v>
       </c>
       <c r="I362" t="n">
-        <v>1233768</v>
+        <v>1232498</v>
       </c>
       <c r="J362" t="inlineStr">
         <is>
@@ -19104,10 +19104,10 @@
         </is>
       </c>
       <c r="K362" t="n">
-        <v>0.04597030716955031</v>
+        <v>0.04489361990735397</v>
       </c>
       <c r="L362" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="363">
@@ -20076,7 +20076,7 @@
         <v>6</v>
       </c>
       <c r="I381" t="n">
-        <v>258998</v>
+        <v>257952</v>
       </c>
       <c r="J381" t="inlineStr">
         <is>
@@ -20084,10 +20084,10 @@
         </is>
       </c>
       <c r="K381" t="n">
-        <v>0.1066635332322088</v>
+        <v>0.1021941162646613</v>
       </c>
       <c r="L381" t="n">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="382">
@@ -21056,7 +21056,7 @@
         <v>6</v>
       </c>
       <c r="I400" t="n">
-        <v>25484</v>
+        <v>25352</v>
       </c>
       <c r="J400" t="inlineStr">
         <is>
@@ -21064,7 +21064,7 @@
         </is>
       </c>
       <c r="K400" t="n">
-        <v>-0.1001094671422014</v>
+        <v>-0.1047706486810975</v>
       </c>
       <c r="L400" t="n">
         <v>1</v>
@@ -22036,7 +22036,7 @@
         <v>6</v>
       </c>
       <c r="I419" t="n">
-        <v>207531</v>
+        <v>206589</v>
       </c>
       <c r="J419" t="inlineStr">
         <is>
@@ -22044,10 +22044,10 @@
         </is>
       </c>
       <c r="K419" t="n">
-        <v>0.07211824085219387</v>
+        <v>0.06725180941360009</v>
       </c>
       <c r="L419" t="n">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="420">
@@ -23016,7 +23016,7 @@
         <v>6</v>
       </c>
       <c r="I438" t="n">
-        <v>406005</v>
+        <v>406224</v>
       </c>
       <c r="J438" t="inlineStr">
         <is>
@@ -23024,10 +23024,10 @@
         </is>
       </c>
       <c r="K438" t="n">
-        <v>0.02483296185699468</v>
+        <v>0.02538575903596207</v>
       </c>
       <c r="L438" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="439">
@@ -23996,7 +23996,7 @@
         <v>6</v>
       </c>
       <c r="I457" t="n">
-        <v>6264268</v>
+        <v>6265112</v>
       </c>
       <c r="J457" t="inlineStr">
         <is>
@@ -24004,10 +24004,10 @@
         </is>
       </c>
       <c r="K457" t="n">
-        <v>0.01892295147749712</v>
+        <v>0.01906023343463037</v>
       </c>
       <c r="L457" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
     </row>
     <row r="458">
@@ -24976,7 +24976,7 @@
         <v>6</v>
       </c>
       <c r="I476" t="n">
-        <v>64593</v>
+        <v>64707</v>
       </c>
       <c r="J476" t="inlineStr">
         <is>
@@ -24984,10 +24984,10 @@
         </is>
       </c>
       <c r="K476" t="n">
-        <v>-0.02589353038757347</v>
+        <v>-0.02417433267983715</v>
       </c>
       <c r="L476" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="477">
@@ -25956,7 +25956,7 @@
         <v>6</v>
       </c>
       <c r="I495" t="n">
-        <v>100173</v>
+        <v>97639</v>
       </c>
       <c r="J495" t="inlineStr">
         <is>
@@ -25964,7 +25964,7 @@
         </is>
       </c>
       <c r="K495" t="n">
-        <v>0.2286793656245016</v>
+        <v>0.1975984005691227</v>
       </c>
       <c r="L495" t="n">
         <v>92</v>
@@ -27916,7 +27916,7 @@
         <v>6</v>
       </c>
       <c r="I533" t="n">
-        <v>206565</v>
+        <v>206394</v>
       </c>
       <c r="J533" t="inlineStr">
         <is>
@@ -27924,7 +27924,7 @@
         </is>
       </c>
       <c r="K533" t="n">
-        <v>0.01970647618389409</v>
+        <v>0.01886233604675835</v>
       </c>
       <c r="L533" t="n">
         <v>23</v>
@@ -28896,7 +28896,7 @@
         <v>6</v>
       </c>
       <c r="I552" t="n">
-        <v>117051</v>
+        <v>116769</v>
       </c>
       <c r="J552" t="inlineStr">
         <is>
@@ -28904,10 +28904,10 @@
         </is>
       </c>
       <c r="K552" t="n">
-        <v>0.05534067241892293</v>
+        <v>0.05279813908198316</v>
       </c>
       <c r="L552" t="n">
-        <v>55</v>
+        <v>52</v>
       </c>
     </row>
     <row r="553">
@@ -29876,7 +29876,7 @@
         <v>6</v>
       </c>
       <c r="I571" t="n">
-        <v>271010</v>
+        <v>270994</v>
       </c>
       <c r="J571" t="inlineStr">
         <is>
@@ -29884,10 +29884,10 @@
         </is>
       </c>
       <c r="K571" t="n">
-        <v>0.04288364002986156</v>
+        <v>0.04282206983599246</v>
       </c>
       <c r="L571" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="572">
@@ -30856,7 +30856,7 @@
         <v>6</v>
       </c>
       <c r="I590" t="n">
-        <v>190958</v>
+        <v>191069</v>
       </c>
       <c r="J590" t="inlineStr">
         <is>
@@ -30864,10 +30864,10 @@
         </is>
       </c>
       <c r="K590" t="n">
-        <v>0.03500831982829178</v>
+        <v>0.03560994910541515</v>
       </c>
       <c r="L590" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="591">
@@ -31836,7 +31836,7 @@
         <v>6</v>
       </c>
       <c r="I609" t="n">
-        <v>1752513</v>
+        <v>1754472</v>
       </c>
       <c r="J609" t="inlineStr">
         <is>
@@ -31844,10 +31844,10 @@
         </is>
       </c>
       <c r="K609" t="n">
-        <v>0.07890574835487341</v>
+        <v>0.08011177442202788</v>
       </c>
       <c r="L609" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="610">
@@ -32816,7 +32816,7 @@
         <v>6</v>
       </c>
       <c r="I628" t="n">
-        <v>3124439</v>
+        <v>3124429</v>
       </c>
       <c r="J628" t="inlineStr">
         <is>
@@ -32824,10 +32824,10 @@
         </is>
       </c>
       <c r="K628" t="n">
-        <v>0.06432323628709669</v>
+        <v>0.06431982984121531</v>
       </c>
       <c r="L628" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="629">
@@ -33796,7 +33796,7 @@
         <v>6</v>
       </c>
       <c r="I647" t="n">
-        <v>1503897</v>
+        <v>1503538</v>
       </c>
       <c r="J647" t="inlineStr">
         <is>
@@ -33804,7 +33804,7 @@
         </is>
       </c>
       <c r="K647" t="n">
-        <v>0.07573276796271311</v>
+        <v>0.07547597639806547</v>
       </c>
       <c r="L647" t="n">
         <v>73</v>
@@ -34776,7 +34776,7 @@
         <v>6</v>
       </c>
       <c r="I666" t="n">
-        <v>561659</v>
+        <v>563107</v>
       </c>
       <c r="J666" t="inlineStr">
         <is>
@@ -34784,7 +34784,7 @@
         </is>
       </c>
       <c r="K666" t="n">
-        <v>0.08174023242645667</v>
+        <v>0.08452904175124898</v>
       </c>
       <c r="L666" t="n">
         <v>79</v>
@@ -35756,7 +35756,7 @@
         <v>6</v>
       </c>
       <c r="I685" t="n">
-        <v>527676</v>
+        <v>528370</v>
       </c>
       <c r="J685" t="inlineStr">
         <is>
@@ -35764,10 +35764,10 @@
         </is>
       </c>
       <c r="K685" t="n">
-        <v>0.05404077327804213</v>
+        <v>0.05542704875135329</v>
       </c>
       <c r="L685" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="686">
@@ -36736,7 +36736,7 @@
         <v>6</v>
       </c>
       <c r="I704" t="n">
-        <v>110779</v>
+        <v>111643</v>
       </c>
       <c r="J704" t="inlineStr">
         <is>
@@ -36744,10 +36744,10 @@
         </is>
       </c>
       <c r="K704" t="n">
-        <v>0.05145314072021101</v>
+        <v>0.05965375196947553</v>
       </c>
       <c r="L704" t="n">
-        <v>51</v>
+        <v>61</v>
       </c>
     </row>
     <row r="705">
@@ -37716,7 +37716,7 @@
         <v>6</v>
       </c>
       <c r="I723" t="n">
-        <v>104570</v>
+        <v>104515</v>
       </c>
       <c r="J723" t="inlineStr">
         <is>
@@ -37724,7 +37724,7 @@
         </is>
       </c>
       <c r="K723" t="n">
-        <v>0.07042686047701907</v>
+        <v>0.06986385505169412</v>
       </c>
       <c r="L723" t="n">
         <v>70</v>
@@ -38696,7 +38696,7 @@
         <v>6</v>
       </c>
       <c r="I742" t="n">
-        <v>128047</v>
+        <v>127988</v>
       </c>
       <c r="J742" t="inlineStr">
         <is>
@@ -38704,10 +38704,10 @@
         </is>
       </c>
       <c r="K742" t="n">
-        <v>0.0650170506529153</v>
+        <v>0.06452632454462282</v>
       </c>
       <c r="L742" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="743">
@@ -39676,7 +39676,7 @@
         <v>6</v>
       </c>
       <c r="I761" t="n">
-        <v>46347</v>
+        <v>46376</v>
       </c>
       <c r="J761" t="inlineStr">
         <is>
@@ -39684,10 +39684,10 @@
         </is>
       </c>
       <c r="K761" t="n">
-        <v>0.02139897743300434</v>
+        <v>0.0220380818053596</v>
       </c>
       <c r="L761" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="762">
@@ -40656,7 +40656,7 @@
         <v>6</v>
       </c>
       <c r="I780" t="n">
-        <v>141790</v>
+        <v>141879</v>
       </c>
       <c r="J780" t="inlineStr">
         <is>
@@ -40664,10 +40664,10 @@
         </is>
       </c>
       <c r="K780" t="n">
-        <v>0.01969780871766469</v>
+        <v>0.02033786164788465</v>
       </c>
       <c r="L780" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="781">
@@ -41636,7 +41636,7 @@
         <v>6</v>
       </c>
       <c r="I799" t="n">
-        <v>411178</v>
+        <v>411234</v>
       </c>
       <c r="J799" t="inlineStr">
         <is>
@@ -41644,7 +41644,7 @@
         </is>
       </c>
       <c r="K799" t="n">
-        <v>-0.08186610873055389</v>
+        <v>-0.08174106435096384</v>
       </c>
       <c r="L799" t="n">
         <v>2</v>
@@ -42616,7 +42616,7 @@
         <v>6</v>
       </c>
       <c r="I818" t="n">
-        <v>8655</v>
+        <v>8670</v>
       </c>
       <c r="J818" t="inlineStr">
         <is>
@@ -42624,10 +42624,10 @@
         </is>
       </c>
       <c r="K818" t="n">
-        <v>0.01429743349349577</v>
+        <v>0.01605531466072896</v>
       </c>
       <c r="L818" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="819">
@@ -43596,7 +43596,7 @@
         <v>6</v>
       </c>
       <c r="I837" t="n">
-        <v>126500</v>
+        <v>126605</v>
       </c>
       <c r="J837" t="inlineStr">
         <is>
@@ -43604,10 +43604,10 @@
         </is>
       </c>
       <c r="K837" t="n">
-        <v>0.02814600486032659</v>
+        <v>0.02899940668254275</v>
       </c>
       <c r="L837" t="n">
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
     <row r="838">
@@ -44576,7 +44576,7 @@
         <v>6</v>
       </c>
       <c r="I856" t="n">
-        <v>371827</v>
+        <v>362271</v>
       </c>
       <c r="J856" t="inlineStr">
         <is>
@@ -44584,10 +44584,10 @@
         </is>
       </c>
       <c r="K856" t="n">
-        <v>0.02960665679039698</v>
+        <v>0.003145638057790112</v>
       </c>
       <c r="L856" t="n">
-        <v>35</v>
+        <v>15</v>
       </c>
     </row>
     <row r="857">
@@ -45556,7 +45556,7 @@
         <v>6</v>
       </c>
       <c r="I875" t="n">
-        <v>4096084</v>
+        <v>4096664</v>
       </c>
       <c r="J875" t="inlineStr">
         <is>
@@ -45564,10 +45564,10 @@
         </is>
       </c>
       <c r="K875" t="n">
-        <v>0.02243316130050022</v>
+        <v>0.02257793646467032</v>
       </c>
       <c r="L875" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="876">
@@ -46536,7 +46536,7 @@
         <v>6</v>
       </c>
       <c r="I894" t="n">
-        <v>63970</v>
+        <v>63345</v>
       </c>
       <c r="J894" t="inlineStr">
         <is>
@@ -46544,10 +46544,10 @@
         </is>
       </c>
       <c r="K894" t="n">
-        <v>0.05779247622984696</v>
+        <v>0.04745762711864399</v>
       </c>
       <c r="L894" t="n">
-        <v>57</v>
+        <v>49</v>
       </c>
     </row>
     <row r="895">
@@ -47516,7 +47516,7 @@
         <v>6</v>
       </c>
       <c r="I913" t="n">
-        <v>119259</v>
+        <v>119415</v>
       </c>
       <c r="J913" t="inlineStr">
         <is>
@@ -47524,10 +47524,10 @@
         </is>
       </c>
       <c r="K913" t="n">
-        <v>0.05318979829736126</v>
+        <v>0.05456745204705227</v>
       </c>
       <c r="L913" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="914">
@@ -48496,7 +48496,7 @@
         <v>6</v>
       </c>
       <c r="I932" t="n">
-        <v>388428</v>
+        <v>386960</v>
       </c>
       <c r="J932" t="inlineStr">
         <is>
@@ -48504,7 +48504,7 @@
         </is>
       </c>
       <c r="K932" t="n">
-        <v>-0.0259738305757975</v>
+        <v>-0.02965500293390444</v>
       </c>
       <c r="L932" t="n">
         <v>6</v>
@@ -49476,7 +49476,7 @@
         <v>6</v>
       </c>
       <c r="I951" t="n">
-        <v>209409</v>
+        <v>209676</v>
       </c>
       <c r="J951" t="inlineStr">
         <is>
@@ -49484,7 +49484,7 @@
         </is>
       </c>
       <c r="K951" t="n">
-        <v>-0.05500500907047901</v>
+        <v>-0.05380012454986061</v>
       </c>
       <c r="L951" t="n">
         <v>3</v>
@@ -50456,7 +50456,7 @@
         <v>6</v>
       </c>
       <c r="I970" t="n">
-        <v>248616</v>
+        <v>250934</v>
       </c>
       <c r="J970" t="inlineStr">
         <is>
@@ -50464,10 +50464,10 @@
         </is>
       </c>
       <c r="K970" t="n">
-        <v>0.09850081520658538</v>
+        <v>0.1087428144731202</v>
       </c>
       <c r="L970" t="n">
-        <v>83</v>
+        <v>86</v>
       </c>
     </row>
     <row r="971">
@@ -51436,7 +51436,7 @@
         <v>6</v>
       </c>
       <c r="I989" t="n">
-        <v>117104</v>
+        <v>117205</v>
       </c>
       <c r="J989" t="inlineStr">
         <is>
@@ -51444,10 +51444,10 @@
         </is>
       </c>
       <c r="K989" t="n">
-        <v>0.001933640206026821</v>
+        <v>0.002797789147658269</v>
       </c>
       <c r="L989" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="990">
@@ -52416,7 +52416,7 @@
         <v>6</v>
       </c>
       <c r="I1008" t="n">
-        <v>478020</v>
+        <v>480611</v>
       </c>
       <c r="J1008" t="inlineStr">
         <is>
@@ -52424,10 +52424,10 @@
         </is>
       </c>
       <c r="K1008" t="n">
-        <v>0.0876722739363216</v>
+        <v>0.09356775709972265</v>
       </c>
       <c r="L1008" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="1009">
@@ -53396,7 +53396,7 @@
         <v>6</v>
       </c>
       <c r="I1027" t="n">
-        <v>203707</v>
+        <v>203728</v>
       </c>
       <c r="J1027" t="inlineStr">
         <is>
@@ -53404,10 +53404,10 @@
         </is>
       </c>
       <c r="K1027" t="n">
-        <v>0.0380080306550894</v>
+        <v>0.03811503811503814</v>
       </c>
       <c r="L1027" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="1028">
@@ -54376,7 +54376,7 @@
         <v>6</v>
       </c>
       <c r="I1046" t="n">
-        <v>107808</v>
+        <v>108566</v>
       </c>
       <c r="J1046" t="inlineStr">
         <is>
@@ -54384,10 +54384,10 @@
         </is>
       </c>
       <c r="K1046" t="n">
-        <v>0.04982909894732734</v>
+        <v>0.05721046635050775</v>
       </c>
       <c r="L1046" t="n">
-        <v>49</v>
+        <v>58</v>
       </c>
     </row>
     <row r="1047">
@@ -55356,7 +55356,7 @@
         <v>6</v>
       </c>
       <c r="I1065" t="n">
-        <v>1589069</v>
+        <v>1589572</v>
       </c>
       <c r="J1065" t="inlineStr">
         <is>
@@ -55364,10 +55364,10 @@
         </is>
       </c>
       <c r="K1065" t="n">
-        <v>0.1002979469151797</v>
+        <v>0.1006462325259985</v>
       </c>
       <c r="L1065" t="n">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="1066">
@@ -57316,7 +57316,7 @@
         <v>6</v>
       </c>
       <c r="I1103" t="n">
-        <v>2371746</v>
+        <v>2371738</v>
       </c>
       <c r="J1103" t="inlineStr">
         <is>
@@ -57324,7 +57324,7 @@
         </is>
       </c>
       <c r="K1103" t="n">
-        <v>0.06605435391850634</v>
+        <v>0.06605075807188898</v>
       </c>
       <c r="L1103" t="n">
         <v>65</v>
@@ -58296,7 +58296,7 @@
         <v>6</v>
       </c>
       <c r="I1122" t="n">
-        <v>19928167</v>
+        <v>19938425</v>
       </c>
       <c r="J1122" t="inlineStr">
         <is>
@@ -58304,10 +58304,10 @@
         </is>
       </c>
       <c r="K1122" t="n">
-        <v>0.05278570902922586</v>
+        <v>0.05332762920699352</v>
       </c>
       <c r="L1122" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="1123">
@@ -59276,7 +59276,7 @@
         <v>6</v>
       </c>
       <c r="I1141" t="n">
-        <v>230769</v>
+        <v>232744</v>
       </c>
       <c r="J1141" t="inlineStr">
         <is>
@@ -59284,10 +59284,10 @@
         </is>
       </c>
       <c r="K1141" t="n">
-        <v>0.0607874232917327</v>
+        <v>0.06986600473465265</v>
       </c>
       <c r="L1141" t="n">
-        <v>61</v>
+        <v>71</v>
       </c>
     </row>
     <row r="1142">
@@ -60256,7 +60256,7 @@
         <v>6</v>
       </c>
       <c r="I1160" t="n">
-        <v>692939</v>
+        <v>693016</v>
       </c>
       <c r="J1160" t="inlineStr">
         <is>
@@ -60264,7 +60264,7 @@
         </is>
       </c>
       <c r="K1160" t="n">
-        <v>0.08093027463973623</v>
+        <v>0.08105038857638469</v>
       </c>
       <c r="L1160" t="n">
         <v>77</v>
@@ -61236,7 +61236,7 @@
         <v>6</v>
       </c>
       <c r="I1179" t="n">
-        <v>802180</v>
+        <v>805662</v>
       </c>
       <c r="J1179" t="inlineStr">
         <is>
@@ -61244,10 +61244,10 @@
         </is>
       </c>
       <c r="K1179" t="n">
-        <v>0.08878974649921356</v>
+        <v>0.09351582530610258</v>
       </c>
       <c r="L1179" t="n">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="1180">
@@ -62216,7 +62216,7 @@
         <v>6</v>
       </c>
       <c r="I1198" t="n">
-        <v>1198619</v>
+        <v>1197344</v>
       </c>
       <c r="J1198" t="inlineStr">
         <is>
@@ -62224,10 +62224,10 @@
         </is>
       </c>
       <c r="K1198" t="n">
-        <v>0.04520487382486071</v>
+        <v>0.04409306413877467</v>
       </c>
       <c r="L1198" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="1199">
@@ -63196,7 +63196,7 @@
         <v>6</v>
       </c>
       <c r="I1217" t="n">
-        <v>599452</v>
+        <v>597467</v>
       </c>
       <c r="J1217" t="inlineStr">
         <is>
@@ -63204,10 +63204,10 @@
         </is>
       </c>
       <c r="K1217" t="n">
-        <v>0.1223065761759887</v>
+        <v>0.1185902176456821</v>
       </c>
       <c r="L1217" t="n">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="1218">
@@ -64176,7 +64176,7 @@
         <v>6</v>
       </c>
       <c r="I1236" t="n">
-        <v>281679</v>
+        <v>282188</v>
       </c>
       <c r="J1236" t="inlineStr">
         <is>
@@ -64184,7 +64184,7 @@
         </is>
       </c>
       <c r="K1236" t="n">
-        <v>0.10043755127554</v>
+        <v>0.1024260655545572</v>
       </c>
       <c r="L1236" t="n">
         <v>85</v>
@@ -65156,7 +65156,7 @@
         <v>6</v>
       </c>
       <c r="I1255" t="n">
-        <v>17553</v>
+        <v>17384</v>
       </c>
       <c r="J1255" t="inlineStr">
         <is>
@@ -65164,10 +65164,10 @@
         </is>
       </c>
       <c r="K1255" t="n">
-        <v>0.02105753010296074</v>
+        <v>0.01122680472340187</v>
       </c>
       <c r="L1255" t="n">
-        <v>24</v>
+        <v>17</v>
       </c>
     </row>
     <row r="1256">
@@ -66136,7 +66136,7 @@
         <v>6</v>
       </c>
       <c r="I1274" t="n">
-        <v>294897</v>
+        <v>292100</v>
       </c>
       <c r="J1274" t="inlineStr">
         <is>
@@ -66144,7 +66144,7 @@
         </is>
       </c>
       <c r="K1274" t="n">
-        <v>0.1519189078338314</v>
+        <v>0.1409933399738286</v>
       </c>
       <c r="L1274" t="n">
         <v>91</v>
@@ -67116,7 +67116,7 @@
         <v>6</v>
       </c>
       <c r="I1293" t="n">
-        <v>30998</v>
+        <v>31050</v>
       </c>
       <c r="J1293" t="inlineStr">
         <is>
@@ -67124,10 +67124,10 @@
         </is>
       </c>
       <c r="K1293" t="n">
-        <v>0.05784390676722517</v>
+        <v>0.05961846909872714</v>
       </c>
       <c r="L1293" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="1294">
@@ -68096,7 +68096,7 @@
         <v>6</v>
       </c>
       <c r="I1312" t="n">
-        <v>314725</v>
+        <v>315071</v>
       </c>
       <c r="J1312" t="inlineStr">
         <is>
@@ -68104,10 +68104,10 @@
         </is>
       </c>
       <c r="K1312" t="n">
-        <v>0.03824064024702034</v>
+        <v>0.03938205342209522</v>
       </c>
       <c r="L1312" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
     </row>
     <row r="1313">
@@ -69076,7 +69076,7 @@
         <v>6</v>
       </c>
       <c r="I1331" t="n">
-        <v>301421</v>
+        <v>295114</v>
       </c>
       <c r="J1331" t="inlineStr">
         <is>
@@ -69084,10 +69084,10 @@
         </is>
       </c>
       <c r="K1331" t="n">
-        <v>0.07898909989081981</v>
+        <v>0.05641209214082443</v>
       </c>
       <c r="L1331" t="n">
-        <v>76</v>
+        <v>57</v>
       </c>
     </row>
     <row r="1332">
@@ -70056,7 +70056,7 @@
         <v>6</v>
       </c>
       <c r="I1350" t="n">
-        <v>13663899</v>
+        <v>13673312</v>
       </c>
       <c r="J1350" t="inlineStr">
         <is>
@@ -70064,7 +70064,7 @@
         </is>
       </c>
       <c r="K1350" t="n">
-        <v>0.06907433939730812</v>
+        <v>0.06981082001362027</v>
       </c>
       <c r="L1350" t="n">
         <v>69</v>
@@ -71036,7 +71036,7 @@
         <v>6</v>
       </c>
       <c r="I1369" t="n">
-        <v>335272</v>
+        <v>338669</v>
       </c>
       <c r="J1369" t="inlineStr">
         <is>
@@ -71044,10 +71044,10 @@
         </is>
       </c>
       <c r="K1369" t="n">
-        <v>0.06751064256580563</v>
+        <v>0.07832673711827653</v>
       </c>
       <c r="L1369" t="n">
-        <v>67</v>
+        <v>75</v>
       </c>
     </row>
     <row r="1370">
@@ -72016,7 +72016,7 @@
         <v>6</v>
       </c>
       <c r="I1388" t="n">
-        <v>122074</v>
+        <v>122262</v>
       </c>
       <c r="J1388" t="inlineStr">
         <is>
@@ -72024,10 +72024,10 @@
         </is>
       </c>
       <c r="K1388" t="n">
-        <v>0.0217791616445695</v>
+        <v>0.02335275210928089</v>
       </c>
       <c r="L1388" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
     </row>
     <row r="1389">
@@ -72996,7 +72996,7 @@
         <v>6</v>
       </c>
       <c r="I1407" t="n">
-        <v>96522</v>
+        <v>96492</v>
       </c>
       <c r="J1407" t="inlineStr">
         <is>
@@ -73004,7 +73004,7 @@
         </is>
       </c>
       <c r="K1407" t="n">
-        <v>0.05654800998292386</v>
+        <v>0.05621962432680938</v>
       </c>
       <c r="L1407" t="n">
         <v>56</v>
@@ -73976,7 +73976,7 @@
         <v>6</v>
       </c>
       <c r="I1426" t="n">
-        <v>34782</v>
+        <v>34808</v>
       </c>
       <c r="J1426" t="inlineStr">
         <is>
@@ -73984,10 +73984,10 @@
         </is>
       </c>
       <c r="K1426" t="n">
-        <v>0.01532533496803579</v>
+        <v>0.01608430393788129</v>
       </c>
       <c r="L1426" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="1427">
@@ -74956,7 +74956,7 @@
         <v>6</v>
       </c>
       <c r="I1445" t="n">
-        <v>179756</v>
+        <v>180188</v>
       </c>
       <c r="J1445" t="inlineStr">
         <is>
@@ -74964,7 +74964,7 @@
         </is>
       </c>
       <c r="K1445" t="n">
-        <v>-0.008226343056712659</v>
+        <v>-0.00584285533001927</v>
       </c>
       <c r="L1445" t="n">
         <v>10</v>
@@ -75936,7 +75936,7 @@
         <v>6</v>
       </c>
       <c r="I1464" t="n">
-        <v>354381</v>
+        <v>354114</v>
       </c>
       <c r="J1464" t="inlineStr">
         <is>
@@ -75944,7 +75944,7 @@
         </is>
       </c>
       <c r="K1464" t="n">
-        <v>0.03941726158701475</v>
+        <v>0.03863413718462372</v>
       </c>
       <c r="L1464" t="n">
         <v>42</v>
@@ -76916,7 +76916,7 @@
         <v>6</v>
       </c>
       <c r="I1483" t="n">
-        <v>721310</v>
+        <v>721307</v>
       </c>
       <c r="J1483" t="inlineStr">
         <is>
@@ -76924,10 +76924,10 @@
         </is>
       </c>
       <c r="K1483" t="n">
-        <v>0.05922502749717684</v>
+        <v>0.05922062207498313</v>
       </c>
       <c r="L1483" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="1484">
@@ -77896,7 +77896,7 @@
         <v>6</v>
       </c>
       <c r="I1502" t="n">
-        <v>1257971</v>
+        <v>1257625</v>
       </c>
       <c r="J1502" t="inlineStr">
         <is>
@@ -77904,10 +77904,10 @@
         </is>
       </c>
       <c r="K1502" t="n">
-        <v>0.02720859020944766</v>
+        <v>0.02692606050708357</v>
       </c>
       <c r="L1502" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
     </row>
     <row r="1503">
@@ -78876,7 +78876,7 @@
         <v>6</v>
       </c>
       <c r="I1521" t="n">
-        <v>109678</v>
+        <v>110441</v>
       </c>
       <c r="J1521" t="inlineStr">
         <is>
@@ -78884,10 +78884,10 @@
         </is>
       </c>
       <c r="K1521" t="n">
-        <v>0.05869861096363804</v>
+        <v>0.06606368910296623</v>
       </c>
       <c r="L1521" t="n">
-        <v>59</v>
+        <v>66</v>
       </c>
     </row>
     <row r="1522">
@@ -80836,7 +80836,7 @@
         <v>6</v>
       </c>
       <c r="I1559" t="n">
-        <v>61533</v>
+        <v>61556</v>
       </c>
       <c r="J1559" t="inlineStr">
         <is>
@@ -80844,7 +80844,7 @@
         </is>
       </c>
       <c r="K1559" t="n">
-        <v>0.02495211126842678</v>
+        <v>0.02533522112101272</v>
       </c>
       <c r="L1559" t="n">
         <v>31</v>
@@ -81816,7 +81816,7 @@
         <v>6</v>
       </c>
       <c r="I1578" t="n">
-        <v>59020</v>
+        <v>59062</v>
       </c>
       <c r="J1578" t="inlineStr">
         <is>
@@ -81824,10 +81824,10 @@
         </is>
       </c>
       <c r="K1578" t="n">
-        <v>0.03493020972154026</v>
+        <v>0.03566669004699441</v>
       </c>
       <c r="L1578" t="n">
-        <v>37</v>
+        <v>40</v>
       </c>
     </row>
     <row r="1579">
@@ -82796,7 +82796,7 @@
         <v>6</v>
       </c>
       <c r="I1597" t="n">
-        <v>452475</v>
+        <v>450873</v>
       </c>
       <c r="J1597" t="inlineStr">
         <is>
@@ -82804,10 +82804,10 @@
         </is>
       </c>
       <c r="K1597" t="n">
-        <v>0.02412079181925586</v>
+        <v>0.02049486440117887</v>
       </c>
       <c r="L1597" t="n">
-        <v>29</v>
+        <v>26</v>
       </c>
     </row>
     <row r="1598">
@@ -83776,7 +83776,7 @@
         <v>6</v>
       </c>
       <c r="I1616" t="n">
-        <v>405372</v>
+        <v>406008</v>
       </c>
       <c r="J1616" t="inlineStr">
         <is>
@@ -83784,10 +83784,10 @@
         </is>
       </c>
       <c r="K1616" t="n">
-        <v>0.05061385071129965</v>
+        <v>0.05226218954341522</v>
       </c>
       <c r="L1616" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="1617">
@@ -84756,7 +84756,7 @@
         <v>6</v>
       </c>
       <c r="I1635" t="n">
-        <v>83845</v>
+        <v>84376</v>
       </c>
       <c r="J1635" t="inlineStr">
         <is>
@@ -84764,10 +84764,10 @@
         </is>
       </c>
       <c r="K1635" t="n">
-        <v>0.07639869566333735</v>
+        <v>0.08321565203995163</v>
       </c>
       <c r="L1635" t="n">
-        <v>74</v>
+        <v>78</v>
       </c>
     </row>
     <row r="1636">
@@ -85736,7 +85736,7 @@
         <v>6</v>
       </c>
       <c r="I1654" t="n">
-        <v>266369</v>
+        <v>256814</v>
       </c>
       <c r="J1654" t="inlineStr">
         <is>
@@ -85744,10 +85744,10 @@
         </is>
       </c>
       <c r="K1654" t="n">
-        <v>0.06359556304453728</v>
+        <v>0.02544301674639238</v>
       </c>
       <c r="L1654" t="n">
-        <v>62</v>
+        <v>33</v>
       </c>
     </row>
     <row r="1655">
@@ -86716,7 +86716,7 @@
         <v>6</v>
       </c>
       <c r="I1673" t="n">
-        <v>7196</v>
+        <v>7022</v>
       </c>
       <c r="J1673" t="inlineStr">
         <is>
@@ -86724,7 +86724,7 @@
         </is>
       </c>
       <c r="K1673" t="n">
-        <v>0.1504396482813748</v>
+        <v>0.1226219024780175</v>
       </c>
       <c r="L1673" t="n">
         <v>90</v>
@@ -87696,7 +87696,7 @@
         <v>6</v>
       </c>
       <c r="I1692" t="n">
-        <v>238125</v>
+        <v>238241</v>
       </c>
       <c r="J1692" t="inlineStr">
         <is>
@@ -87704,10 +87704,10 @@
         </is>
       </c>
       <c r="K1692" t="n">
-        <v>0.02596305886712136</v>
+        <v>0.02646284559606027</v>
       </c>
       <c r="L1692" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="1693">
@@ -88676,7 +88676,7 @@
         <v>6</v>
       </c>
       <c r="I1711" t="n">
-        <v>97131</v>
+        <v>97264</v>
       </c>
       <c r="J1711" t="inlineStr">
         <is>
@@ -88684,7 +88684,7 @@
         </is>
       </c>
       <c r="K1711" t="n">
-        <v>-0.01251499562839309</v>
+        <v>-0.01116284744108498</v>
       </c>
       <c r="L1711" t="n">
         <v>9</v>
@@ -89656,7 +89656,7 @@
         <v>6</v>
       </c>
       <c r="I1730" t="n">
-        <v>137920</v>
+        <v>137836</v>
       </c>
       <c r="J1730" t="inlineStr">
         <is>
@@ -89664,10 +89664,10 @@
         </is>
       </c>
       <c r="K1730" t="n">
-        <v>0.06609775139330143</v>
+        <v>0.06544844591826471</v>
       </c>
       <c r="L1730" t="n">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="1731">

</xml_diff>